<commit_message>
M7: Dashboard & Analytics
</commit_message>
<xml_diff>
--- a/dbStructure.xlsx
+++ b/dbStructure.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="7" r:id="rId1"/>
@@ -14,13 +14,14 @@
     <sheet name="learning_history" sheetId="4" r:id="rId5"/>
     <sheet name="user_streaks" sheetId="5" r:id="rId6"/>
     <sheet name="user_badges" sheetId="6" r:id="rId7"/>
+    <sheet name="all tables" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="116">
   <si>
     <t>Tên trường (Column)</t>
   </si>
@@ -2645,4 +2646,684 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D80"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="30.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="17.5">
+      <c r="A1" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="8"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1"/>
+    <row r="8" spans="1:4" ht="15" thickBot="1">
+      <c r="A8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" thickBot="1">
+      <c r="A9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" thickBot="1">
+      <c r="A10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1">
+      <c r="A11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" thickBot="1">
+      <c r="A12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" thickBot="1">
+      <c r="A13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17.5">
+      <c r="A15" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="8"/>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="8"/>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1"/>
+    <row r="21" spans="1:4" ht="15" thickBot="1">
+      <c r="A21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1">
+      <c r="A22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" thickBot="1">
+      <c r="A23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" thickBot="1">
+      <c r="A24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" thickBot="1">
+      <c r="A28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="17.5">
+      <c r="A30" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="8"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="8"/>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" thickBot="1"/>
+    <row r="36" spans="1:4" ht="15" thickBot="1">
+      <c r="A36" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" thickBot="1">
+      <c r="A38" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" thickBot="1">
+      <c r="A39" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" thickBot="1">
+      <c r="A40" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15" thickBot="1">
+      <c r="A41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A42" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="17.5">
+      <c r="A44" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="8"/>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="8"/>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15" thickBot="1"/>
+    <row r="50" spans="1:4" ht="15" thickBot="1">
+      <c r="A50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" thickBot="1">
+      <c r="A51" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15" thickBot="1">
+      <c r="A52" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A53" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" thickBot="1">
+      <c r="A54" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A55" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A56" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="17.5">
+      <c r="A58" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="8"/>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="8"/>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="15" thickBot="1"/>
+    <row r="64" spans="1:4" ht="15" thickBot="1">
+      <c r="A64" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" thickBot="1">
+      <c r="A65" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A66" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15" thickBot="1">
+      <c r="A67" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A68" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="17.5">
+      <c r="A70" s="10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="8"/>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="8"/>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15" thickBot="1"/>
+    <row r="76" spans="1:4" ht="15" thickBot="1">
+      <c r="A76" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="15" thickBot="1">
+      <c r="A77" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="15" thickBot="1">
+      <c r="A78" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="29.5" thickBot="1">
+      <c r="A79" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="15" thickBot="1">
+      <c r="A80" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update project source code and system design
</commit_message>
<xml_diff>
--- a/dbStructure.xlsx
+++ b/dbStructure.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="7" r:id="rId1"/>
@@ -14,13 +14,14 @@
     <sheet name="learning_history" sheetId="4" r:id="rId5"/>
     <sheet name="user_streaks" sheetId="5" r:id="rId6"/>
     <sheet name="user_badges" sheetId="6" r:id="rId7"/>
+    <sheet name="all tables" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="116">
   <si>
     <t>Tên trường (Column)</t>
   </si>
@@ -2645,4 +2646,684 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D80"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="30.1796875" customWidth="1"/>
+    <col min="2" max="2" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="17.5">
+      <c r="A1" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="8"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1"/>
+    <row r="8" spans="1:4" ht="15" thickBot="1">
+      <c r="A8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" thickBot="1">
+      <c r="A9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" thickBot="1">
+      <c r="A10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1">
+      <c r="A11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" thickBot="1">
+      <c r="A12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" thickBot="1">
+      <c r="A13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="17.5">
+      <c r="A15" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="8"/>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="8"/>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1"/>
+    <row r="21" spans="1:4" ht="15" thickBot="1">
+      <c r="A21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1">
+      <c r="A22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" thickBot="1">
+      <c r="A23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" thickBot="1">
+      <c r="A24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" thickBot="1">
+      <c r="A28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="17.5">
+      <c r="A30" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="8"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="8"/>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" thickBot="1"/>
+    <row r="36" spans="1:4" ht="15" thickBot="1">
+      <c r="A36" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" thickBot="1">
+      <c r="A38" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" thickBot="1">
+      <c r="A39" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" thickBot="1">
+      <c r="A40" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15" thickBot="1">
+      <c r="A41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A42" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="17.5">
+      <c r="A44" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="8"/>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="8"/>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="15" thickBot="1"/>
+    <row r="50" spans="1:4" ht="15" thickBot="1">
+      <c r="A50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="15" thickBot="1">
+      <c r="A51" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15" thickBot="1">
+      <c r="A52" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A53" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="15" thickBot="1">
+      <c r="A54" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A55" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A56" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="17.5">
+      <c r="A58" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="8"/>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="8"/>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="15" thickBot="1"/>
+    <row r="64" spans="1:4" ht="15" thickBot="1">
+      <c r="A64" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" thickBot="1">
+      <c r="A65" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A66" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15" thickBot="1">
+      <c r="A67" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="28.5" thickBot="1">
+      <c r="A68" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="17.5">
+      <c r="A70" s="10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="8"/>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="8"/>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15" thickBot="1"/>
+    <row r="76" spans="1:4" ht="15" thickBot="1">
+      <c r="A76" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="15" thickBot="1">
+      <c r="A77" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="15" thickBot="1">
+      <c r="A78" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="29.5" thickBot="1">
+      <c r="A79" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="15" thickBot="1">
+      <c r="A80" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>